<commit_message>
v5: auditoría de seguridad cerrada (#1–#10) y consolidación del proyecto
- Corrige los 10 hallazgos de la auditoría: auth en todos los endpoints
  (#10), dinero en Numeric(12,2) con conversión en el lifespan (#6),
  cuotas MSI exactas (#7), rate limiter reactivado (#5), 401 con aviso
  de sesión expirada en req() (#9), limpieza de JS duplicado (#8) y
  correcciones de UI (#1-#4).
- Nuevos módulos y recursos: auth.py con require_role, dashboard.js,
  contabilidad.js, conteo.js, migración Alembic de contabilidad/OC y
  scripts de mantenimiento (snapshot.py, migraciones, actualización de precios).
- docker-compose: elimina DATABASE_URL con credenciales en claro (ahora
  vía .env), corre sin --reload, fija TZ America/Mexico_City y monta ./backups.
- Higiene del repo: deja de versionar .env y los .pyc de la app, agrega
  .gitignore (venv, backups, zip, postgres_data).
- Documentación: DOCUMENTACION_MAESTRA.md con bitácora y cierre formal
  de la auditoría.
</commit_message>
<xml_diff>
--- a/backend/precios.xlsx
+++ b/backend/precios.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\35 - Docker Compose\01 - App Inventario\inventario_app\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\35 - Docker Compose\01 - App Inventario\inventario_app_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B3F1944-354E-48C7-8793-B949889305F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C68117-5F82-4388-A8CF-04F67329E6DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{91A8A681-0F66-4DED-BEC0-BB0A66BBBA7D}"/>
   </bookViews>
@@ -238,7 +238,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -253,13 +253,45 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -275,15 +307,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -626,54 +683,54 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="1" t="s">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1" t="s">
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="U2" s="1"/>
-      <c r="V2" s="1"/>
-      <c r="W2" s="1"/>
-      <c r="X2" s="1"/>
-      <c r="Y2" s="1"/>
-      <c r="Z2" s="1"/>
-      <c r="AA2" s="1"/>
-      <c r="AB2" s="1"/>
-      <c r="AC2" s="1"/>
-      <c r="AD2" s="1"/>
-      <c r="AE2" s="1"/>
-      <c r="AF2" s="1"/>
-      <c r="AG2" s="1"/>
-      <c r="AH2" s="1"/>
-      <c r="AI2" s="1"/>
-      <c r="AJ2" s="1"/>
-      <c r="AK2" s="1"/>
-      <c r="AL2" s="1"/>
-      <c r="AM2" s="1"/>
-      <c r="AN2" s="1"/>
-      <c r="AO2" s="1"/>
-      <c r="AP2" s="1"/>
-      <c r="AQ2" s="1"/>
-      <c r="AR2" s="1"/>
-      <c r="AS2" s="1"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
+      <c r="X2" s="4"/>
+      <c r="Y2" s="4"/>
+      <c r="Z2" s="4"/>
+      <c r="AA2" s="4"/>
+      <c r="AB2" s="4"/>
+      <c r="AC2" s="4"/>
+      <c r="AD2" s="4"/>
+      <c r="AE2" s="4"/>
+      <c r="AF2" s="4"/>
+      <c r="AG2" s="4"/>
+      <c r="AH2" s="4"/>
+      <c r="AI2" s="4"/>
+      <c r="AJ2" s="4"/>
+      <c r="AK2" s="4"/>
+      <c r="AL2" s="4"/>
+      <c r="AM2" s="4"/>
+      <c r="AN2" s="4"/>
+      <c r="AO2" s="4"/>
+      <c r="AP2" s="4"/>
+      <c r="AQ2" s="4"/>
+      <c r="AR2" s="4"/>
+      <c r="AS2" s="4"/>
     </row>
     <row r="3" spans="2:45" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
@@ -1724,732 +1781,774 @@
       </c>
     </row>
     <row r="13" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="F13" s="1" t="s">
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="N13" s="1" t="s">
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="N13" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="1"/>
+      <c r="O13" s="13"/>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="13"/>
+      <c r="R13" s="13"/>
+      <c r="S13" s="13"/>
+      <c r="T13" s="13"/>
     </row>
     <row r="14" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="C14" t="s">
+      <c r="C14" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="L14" t="s">
+      <c r="L14" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="N14" t="s">
+      <c r="N14" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="O14" t="s">
+      <c r="O14" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="P14" t="s">
+      <c r="P14" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="Q14" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="R14" t="s">
+      <c r="R14" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="S14" t="s">
+      <c r="S14" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="T14" t="s">
+      <c r="T14" s="14" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="15" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="C15" t="s">
-        <v>50</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="C15" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G15" s="3">
+      <c r="F15" s="5"/>
+      <c r="G15" s="7">
         <v>38.28</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="7">
         <v>38.28</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="7">
         <v>38.28</v>
       </c>
-      <c r="J15" s="3">
+      <c r="J15" s="7">
         <v>38.28</v>
       </c>
-      <c r="K15" s="3">
+      <c r="K15" s="7">
         <v>48.14</v>
       </c>
-      <c r="L15" s="3">
+      <c r="L15" s="7">
         <v>60.32</v>
       </c>
-      <c r="O15" s="3">
+      <c r="N15" s="14"/>
+      <c r="O15" s="15">
         <v>60</v>
       </c>
-      <c r="P15" s="3">
+      <c r="P15" s="15">
         <v>60</v>
       </c>
-      <c r="Q15" s="3">
+      <c r="Q15" s="15">
         <v>60</v>
       </c>
-      <c r="R15" s="3">
+      <c r="R15" s="15">
         <v>60</v>
       </c>
-      <c r="S15" s="3">
+      <c r="S15" s="15">
         <v>75</v>
       </c>
-      <c r="T15" s="3">
+      <c r="T15" s="15">
         <v>94.5</v>
       </c>
     </row>
     <row r="16" spans="2:45" x14ac:dyDescent="0.25">
-      <c r="C16" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="C16" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="3">
+      <c r="F16" s="5"/>
+      <c r="G16" s="7">
         <v>44.08</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="7">
         <v>44.08</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="7">
         <v>44.08</v>
       </c>
-      <c r="J16" s="3">
+      <c r="J16" s="7">
         <v>44.08</v>
       </c>
-      <c r="K16" s="3">
+      <c r="K16" s="7">
         <v>55.1</v>
       </c>
-      <c r="L16" s="3">
+      <c r="L16" s="7">
         <v>69.02</v>
       </c>
-      <c r="O16" s="3">
+      <c r="N16" s="14"/>
+      <c r="O16" s="15">
         <v>65</v>
       </c>
-      <c r="P16" s="3">
+      <c r="P16" s="15">
         <v>65</v>
       </c>
-      <c r="Q16" s="3">
+      <c r="Q16" s="15">
         <v>65</v>
       </c>
-      <c r="R16" s="3">
+      <c r="R16" s="15">
         <v>65</v>
       </c>
-      <c r="S16" s="3">
+      <c r="S16" s="15">
         <v>85</v>
       </c>
-      <c r="T16" s="3">
+      <c r="T16" s="15">
         <v>105</v>
       </c>
     </row>
     <row r="17" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C17" t="s">
-        <v>50</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="C17" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="N17" s="14"/>
+      <c r="O17" s="14"/>
+      <c r="P17" s="14"/>
+      <c r="Q17" s="14"/>
+      <c r="R17" s="14"/>
+      <c r="S17" s="14"/>
+      <c r="T17" s="14"/>
     </row>
     <row r="18" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C18" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="C18" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G18" s="5">
+      <c r="F18" s="5"/>
+      <c r="G18" s="8">
         <v>44.08</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="8">
         <v>44.08</v>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="8">
         <v>44.08</v>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="8">
         <v>44.08</v>
       </c>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5">
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16">
         <v>65</v>
       </c>
-      <c r="P18" s="5">
+      <c r="P18" s="16">
         <v>65</v>
       </c>
-      <c r="Q18" s="5">
+      <c r="Q18" s="16">
         <v>65</v>
       </c>
-      <c r="R18" s="5">
+      <c r="R18" s="16">
         <v>65</v>
       </c>
-      <c r="S18" s="5"/>
-      <c r="T18" s="5"/>
+      <c r="S18" s="16"/>
+      <c r="T18" s="16"/>
     </row>
     <row r="19" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C19" t="s">
-        <v>50</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="C19" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="G19" s="5">
+      <c r="F19" s="5"/>
+      <c r="G19" s="8">
         <v>31.3</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="8">
         <v>31.3</v>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="8">
         <v>31.3</v>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="8">
         <v>31.3</v>
       </c>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5">
-        <v>50</v>
-      </c>
-      <c r="P19" s="5">
-        <v>50</v>
-      </c>
-      <c r="Q19" s="5">
-        <v>50</v>
-      </c>
-      <c r="R19" s="5">
-        <v>50</v>
-      </c>
-      <c r="S19" s="5"/>
-      <c r="T19" s="5"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="16">
+        <v>50</v>
+      </c>
+      <c r="P19" s="16">
+        <v>50</v>
+      </c>
+      <c r="Q19" s="16">
+        <v>50</v>
+      </c>
+      <c r="R19" s="16">
+        <v>50</v>
+      </c>
+      <c r="S19" s="16"/>
+      <c r="T19" s="16"/>
     </row>
     <row r="20" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C20" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="C20" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G20" s="5">
+      <c r="F20" s="5"/>
+      <c r="G20" s="8">
         <v>27.26</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="8">
         <v>27.26</v>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="8">
         <v>27.26</v>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="8">
         <v>27.26</v>
       </c>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5">
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16">
         <v>40</v>
       </c>
-      <c r="P20" s="5">
+      <c r="P20" s="16">
         <v>40</v>
       </c>
-      <c r="Q20" s="5">
+      <c r="Q20" s="16">
         <v>40</v>
       </c>
-      <c r="R20" s="5">
+      <c r="R20" s="16">
         <v>40</v>
       </c>
-      <c r="S20" s="5"/>
-      <c r="T20" s="5"/>
+      <c r="S20" s="16"/>
+      <c r="T20" s="16"/>
     </row>
     <row r="21" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="C21" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="G21" s="5">
+      <c r="F21" s="5"/>
+      <c r="G21" s="8">
         <v>26.68</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="8">
         <v>26.68</v>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="8">
         <v>26.68</v>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="8">
         <v>26.68</v>
       </c>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5">
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="16">
         <v>40</v>
       </c>
-      <c r="P21" s="5">
+      <c r="P21" s="16">
         <v>40</v>
       </c>
-      <c r="Q21" s="5">
+      <c r="Q21" s="16">
         <v>40</v>
       </c>
-      <c r="R21" s="5">
+      <c r="R21" s="16">
         <v>40</v>
       </c>
-      <c r="S21" s="5"/>
-      <c r="T21" s="5"/>
+      <c r="S21" s="16"/>
+      <c r="T21" s="16"/>
     </row>
     <row r="22" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="4"/>
-      <c r="S22" s="4"/>
-      <c r="T22" s="4"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="17"/>
+      <c r="O22" s="17"/>
+      <c r="P22" s="17"/>
+      <c r="Q22" s="17"/>
+      <c r="R22" s="17"/>
+      <c r="S22" s="17"/>
+      <c r="T22" s="17"/>
     </row>
     <row r="26" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="F26" s="1" t="s">
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-      <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
-      <c r="N26" s="1" t="s">
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+      <c r="N26" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
-      <c r="Q26" s="1"/>
-      <c r="R26" s="1"/>
-      <c r="S26" s="1"/>
-      <c r="T26" s="1"/>
+      <c r="O26" s="21"/>
+      <c r="P26" s="21"/>
+      <c r="Q26" s="21"/>
+      <c r="R26" s="21"/>
+      <c r="S26" s="21"/>
+      <c r="T26" s="21"/>
     </row>
     <row r="27" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C27" t="s">
+      <c r="C27" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H27" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="K27" t="s">
+      <c r="K27" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="L27" t="s">
+      <c r="L27" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="N27" t="s">
+      <c r="N27" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="O27" t="s">
+      <c r="O27" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="P27" t="s">
+      <c r="P27" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="Q27" t="s">
+      <c r="Q27" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="R27" t="s">
+      <c r="R27" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="S27" t="s">
+      <c r="S27" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="T27" t="s">
+      <c r="T27" s="18" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="28" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C28" t="s">
-        <v>50</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="C28" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="G28" s="3">
+      <c r="F28" s="10"/>
+      <c r="G28" s="11">
         <v>44.08</v>
       </c>
-      <c r="H28" s="3">
+      <c r="H28" s="11">
         <v>44.08</v>
       </c>
-      <c r="I28" s="3">
+      <c r="I28" s="11">
         <v>44.08</v>
       </c>
-      <c r="J28" s="3">
+      <c r="J28" s="11">
         <v>44.08</v>
       </c>
-      <c r="K28" s="3">
+      <c r="K28" s="11">
         <v>55.1</v>
       </c>
-      <c r="L28" s="3">
+      <c r="L28" s="11">
         <v>69.02</v>
       </c>
-      <c r="O28" s="3">
+      <c r="N28" s="18"/>
+      <c r="O28" s="19">
         <v>60</v>
       </c>
-      <c r="P28" s="3">
+      <c r="P28" s="19">
         <v>60</v>
       </c>
-      <c r="Q28" s="3">
+      <c r="Q28" s="19">
         <v>60</v>
       </c>
-      <c r="R28" s="3">
+      <c r="R28" s="19">
         <v>60</v>
       </c>
-      <c r="S28" s="3">
+      <c r="S28" s="19">
         <v>75</v>
       </c>
-      <c r="T28" s="3">
+      <c r="T28" s="19">
         <v>94.5</v>
       </c>
     </row>
     <row r="29" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C29" t="s">
-        <v>50</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="C29" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="G29" s="3">
+      <c r="F29" s="10"/>
+      <c r="G29" s="11">
         <v>51.04</v>
       </c>
-      <c r="H29" s="3">
+      <c r="H29" s="11">
         <v>51.04</v>
       </c>
-      <c r="I29" s="3">
+      <c r="I29" s="11">
         <v>51.04</v>
       </c>
-      <c r="J29" s="3">
+      <c r="J29" s="11">
         <v>51.04</v>
       </c>
-      <c r="K29" s="3">
+      <c r="K29" s="11">
         <v>63.8</v>
       </c>
-      <c r="L29" s="3">
+      <c r="L29" s="11">
         <v>80.040000000000006</v>
       </c>
-      <c r="O29" s="3">
+      <c r="N29" s="18"/>
+      <c r="O29" s="19">
         <v>65</v>
       </c>
-      <c r="P29" s="3">
+      <c r="P29" s="19">
         <v>65</v>
       </c>
-      <c r="Q29" s="3">
+      <c r="Q29" s="19">
         <v>65</v>
       </c>
-      <c r="R29" s="3">
+      <c r="R29" s="19">
         <v>65</v>
       </c>
-      <c r="S29" s="3">
+      <c r="S29" s="19">
         <v>85</v>
       </c>
-      <c r="T29" s="3">
+      <c r="T29" s="19">
         <v>105</v>
       </c>
     </row>
     <row r="30" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C30" t="s">
-        <v>50</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="C30" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D30" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-      <c r="K30" s="3"/>
-      <c r="L30" s="3"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+      <c r="J30" s="11"/>
+      <c r="K30" s="11"/>
+      <c r="L30" s="11"/>
+      <c r="N30" s="18"/>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
     </row>
     <row r="31" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C31" t="s">
-        <v>50</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="C31" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="G31" s="5">
+      <c r="F31" s="10"/>
+      <c r="G31" s="12">
         <v>51.04</v>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="12">
         <v>51.04</v>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="12">
         <v>51.04</v>
       </c>
-      <c r="J31" s="5">
+      <c r="J31" s="12">
         <v>51.04</v>
       </c>
-      <c r="K31" s="5"/>
-      <c r="L31" s="5"/>
-      <c r="M31" s="5"/>
-      <c r="N31" s="5"/>
-      <c r="O31" s="5">
+      <c r="K31" s="12"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="20"/>
+      <c r="O31" s="20">
         <v>65</v>
       </c>
-      <c r="P31" s="5">
+      <c r="P31" s="20">
         <v>65</v>
       </c>
-      <c r="Q31" s="5">
+      <c r="Q31" s="20">
         <v>65</v>
       </c>
-      <c r="R31" s="5">
+      <c r="R31" s="20">
         <v>65</v>
       </c>
-      <c r="S31" s="5"/>
-      <c r="T31" s="5"/>
+      <c r="S31" s="20"/>
+      <c r="T31" s="20"/>
     </row>
     <row r="32" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C32" t="s">
-        <v>50</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="C32" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D32" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="G32" s="5">
+      <c r="F32" s="10"/>
+      <c r="G32" s="12">
         <v>37.700000000000003</v>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="12">
         <v>37.700000000000003</v>
       </c>
-      <c r="I32" s="5">
+      <c r="I32" s="12">
         <v>37.700000000000003</v>
       </c>
-      <c r="J32" s="5">
+      <c r="J32" s="12">
         <v>37.700000000000003</v>
       </c>
-      <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
-      <c r="M32" s="5"/>
-      <c r="N32" s="5"/>
-      <c r="O32" s="5">
-        <v>50</v>
-      </c>
-      <c r="P32" s="5">
-        <v>50</v>
-      </c>
-      <c r="Q32" s="5">
-        <v>50</v>
-      </c>
-      <c r="R32" s="5">
-        <v>50</v>
-      </c>
-      <c r="S32" s="5"/>
-      <c r="T32" s="5"/>
+      <c r="K32" s="12"/>
+      <c r="L32" s="12"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="20"/>
+      <c r="O32" s="20">
+        <v>50</v>
+      </c>
+      <c r="P32" s="20">
+        <v>50</v>
+      </c>
+      <c r="Q32" s="20">
+        <v>50</v>
+      </c>
+      <c r="R32" s="20">
+        <v>50</v>
+      </c>
+      <c r="S32" s="20"/>
+      <c r="T32" s="20"/>
     </row>
     <row r="33" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C33" t="s">
-        <v>50</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="C33" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="G33" s="5">
+      <c r="F33" s="10"/>
+      <c r="G33" s="12">
         <v>32.479999999999997</v>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="12">
         <v>32.479999999999997</v>
       </c>
-      <c r="I33" s="5">
+      <c r="I33" s="12">
         <v>32.479999999999997</v>
       </c>
-      <c r="J33" s="5">
+      <c r="J33" s="12">
         <v>32.479999999999997</v>
       </c>
-      <c r="K33" s="5"/>
-      <c r="L33" s="5"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="5"/>
-      <c r="O33" s="5">
+      <c r="K33" s="12"/>
+      <c r="L33" s="12"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="20"/>
+      <c r="O33" s="20">
         <v>40</v>
       </c>
-      <c r="P33" s="5">
+      <c r="P33" s="20">
         <v>40</v>
       </c>
-      <c r="Q33" s="5">
+      <c r="Q33" s="20">
         <v>40</v>
       </c>
-      <c r="R33" s="5">
+      <c r="R33" s="20">
         <v>40</v>
       </c>
-      <c r="S33" s="5"/>
-      <c r="T33" s="5"/>
+      <c r="S33" s="20"/>
+      <c r="T33" s="20"/>
     </row>
     <row r="34" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="C34" t="s">
-        <v>50</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="C34" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G34" s="5">
+      <c r="F34" s="10"/>
+      <c r="G34" s="12">
         <v>31.9</v>
       </c>
-      <c r="H34" s="5">
+      <c r="H34" s="12">
         <v>31.9</v>
       </c>
-      <c r="I34" s="5">
+      <c r="I34" s="12">
         <v>31.9</v>
       </c>
-      <c r="J34" s="5">
+      <c r="J34" s="12">
         <v>31.9</v>
       </c>
-      <c r="K34" s="5"/>
-      <c r="L34" s="5"/>
-      <c r="M34" s="5"/>
-      <c r="N34" s="5"/>
-      <c r="O34" s="5">
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="20"/>
+      <c r="O34" s="20">
         <v>40</v>
       </c>
-      <c r="P34" s="5">
+      <c r="P34" s="20">
         <v>40</v>
       </c>
-      <c r="Q34" s="5">
+      <c r="Q34" s="20">
         <v>40</v>
       </c>
-      <c r="R34" s="5">
+      <c r="R34" s="20">
         <v>40</v>
       </c>
-      <c r="S34" s="5"/>
-      <c r="T34" s="5"/>
+      <c r="S34" s="20"/>
+      <c r="T34" s="20"/>
     </row>
     <row r="35" spans="3:20" x14ac:dyDescent="0.25">
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="4"/>
-      <c r="M35" s="4"/>
-      <c r="N35" s="4"/>
-      <c r="O35" s="4"/>
-      <c r="P35" s="4"/>
-      <c r="Q35" s="4"/>
-      <c r="R35" s="4"/>
-      <c r="S35" s="4"/>
-      <c r="T35" s="4"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
+      <c r="P35" s="2"/>
+      <c r="Q35" s="2"/>
+      <c r="R35" s="2"/>
+      <c r="S35" s="2"/>
+      <c r="T35" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2461,6 +2560,6 @@
     <mergeCell ref="N13:T13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>